<commit_message>
added all kaggle notebooks and updated the perf score spreadsheet
</commit_message>
<xml_diff>
--- a/kaggle notebooks/Macro AUROC performance scores.xlsx
+++ b/kaggle notebooks/Macro AUROC performance scores.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Deepshik\Documents\GITHUB\ptbxl-ssl-objectives\kaggle notebooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68EFB063-85A7-4295-8BBA-58EB3764F00C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78781312-E3DF-4C54-95C6-DB54412D011D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13695" xr2:uid="{F3BA4440-4B19-4A03-AF21-B6DEA26C06F7}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="13">
   <si>
     <t>Baseline</t>
   </si>
@@ -64,12 +64,24 @@
   <si>
     <t>Methods</t>
   </si>
+  <si>
+    <t>[seed 22]</t>
+  </si>
+  <si>
+    <t>[seed 54]</t>
+  </si>
+  <si>
+    <t>[seed 71]</t>
+  </si>
+  <si>
+    <t>[mean +/- SD]</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -91,16 +103,43 @@
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-4.9989318521683403E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="12">
+  <borders count="21">
     <border>
       <left/>
       <right/>
@@ -171,33 +210,70 @@
     </border>
     <border>
       <left/>
+      <right/>
+      <top/>
+      <bottom style="thick">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
       <right style="thick">
         <color indexed="64"/>
       </right>
       <top style="thin">
         <color indexed="64"/>
       </top>
-      <bottom/>
+      <bottom style="thick">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thick">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thick">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thick">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thick">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
       <left/>
       <right/>
       <top/>
-      <bottom style="thick">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thick">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thick">
+      <bottom style="thin">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -205,38 +281,96 @@
     <border>
       <left/>
       <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thick">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thick">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thick">
         <color indexed="64"/>
       </right>
       <top/>
       <bottom style="thick">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thick">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thick">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -245,7 +379,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -253,49 +387,88 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -632,259 +805,1072 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A3B2FC2-CB8B-412F-85A4-7FB574126CD9}">
-  <dimension ref="A1:H11"/>
+  <dimension ref="B2:R39"/>
   <sheetFormatPr defaultRowHeight="13.5"/>
   <cols>
-    <col min="1" max="1" width="3.5625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="7.5625" style="1" customWidth="1"/>
-    <col min="4" max="16384" width="9" style="1"/>
+    <col min="1" max="1" width="9" style="1"/>
+    <col min="2" max="2" width="3.5625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="10.5625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="7.5625" style="1" customWidth="1"/>
+    <col min="5" max="10" width="9" style="1"/>
+    <col min="11" max="11" width="3.5625" style="1" customWidth="1"/>
+    <col min="12" max="12" width="10.5625" style="1" customWidth="1"/>
+    <col min="13" max="13" width="7.5625" style="1" customWidth="1"/>
+    <col min="14" max="18" width="10.5625" style="1" customWidth="1"/>
+    <col min="19" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
-      <c r="D1" s="7" t="s">
+    <row r="2" spans="2:18">
+      <c r="B2" s="13"/>
+      <c r="C2" s="23" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="23"/>
+      <c r="G2" s="23"/>
+      <c r="H2" s="23"/>
+      <c r="I2" s="24"/>
+    </row>
+    <row r="3" spans="2:18">
+      <c r="B3" s="14"/>
+      <c r="E3" s="25" t="s">
         <v>7</v>
       </c>
-      <c r="E1" s="7"/>
-      <c r="F1" s="7"/>
-      <c r="G1" s="7"/>
-      <c r="H1" s="7"/>
-    </row>
-    <row r="2" spans="1:8">
-      <c r="D2" s="4">
+      <c r="F3" s="25"/>
+      <c r="G3" s="25"/>
+      <c r="H3" s="25"/>
+      <c r="I3" s="26"/>
+    </row>
+    <row r="4" spans="2:18" ht="13.9" thickBot="1">
+      <c r="B4" s="14"/>
+      <c r="E4" s="12">
         <v>0.01</v>
       </c>
-      <c r="E2" s="4">
+      <c r="F4" s="12">
         <v>0.05</v>
       </c>
-      <c r="F2" s="4">
+      <c r="G4" s="12">
         <v>0.1</v>
       </c>
-      <c r="G2" s="4">
+      <c r="H4" s="12">
         <v>0.25</v>
       </c>
-      <c r="H2" s="4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" ht="13.9" thickBot="1">
-      <c r="A3" s="8" t="s">
+      <c r="I4" s="15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="2:18" ht="14.25" customHeight="1" thickTop="1" thickBot="1">
+      <c r="B5" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="13" t="s">
+      <c r="C5" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="17"/>
-      <c r="D3" s="15">
+      <c r="D5" s="20"/>
+      <c r="E5" s="10">
         <v>0.61799999999999999</v>
       </c>
-      <c r="E3" s="16">
+      <c r="F5" s="11">
         <v>0.78</v>
       </c>
-      <c r="F3" s="16">
+      <c r="G5" s="11">
         <v>0.81799999999999995</v>
       </c>
-      <c r="G3" s="16">
+      <c r="H5" s="11">
         <v>0.83699999999999997</v>
       </c>
-      <c r="H3" s="16">
+      <c r="I5" s="11">
         <v>0.92600000000000005</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="13.9" thickTop="1">
-      <c r="A4" s="8"/>
-      <c r="B4" s="5" t="s">
+    <row r="6" spans="2:18" ht="13.9" thickTop="1">
+      <c r="B6" s="17"/>
+      <c r="C6" s="21" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="11" t="s">
-        <v>1</v>
-      </c>
-      <c r="D4" s="9">
+      <c r="D6" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="E6" s="8">
         <v>0.57799999999999996</v>
       </c>
-      <c r="E4" s="3">
+      <c r="F6" s="9">
         <v>0.65600000000000003</v>
       </c>
-      <c r="F4" s="3">
+      <c r="G6" s="9">
         <v>0.76100000000000001</v>
       </c>
-      <c r="G4" s="3">
+      <c r="H6" s="9">
         <v>0.82599999999999996</v>
       </c>
-      <c r="H4" s="3">
+      <c r="I6" s="9">
         <v>0.91400000000000003</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="13.9" thickBot="1">
-      <c r="A5" s="8"/>
-      <c r="B5" s="13"/>
-      <c r="C5" s="14" t="s">
+    <row r="7" spans="2:18" ht="13.9" thickBot="1">
+      <c r="B7" s="17"/>
+      <c r="C7" s="19"/>
+      <c r="D7" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="15">
+      <c r="E7" s="5">
         <v>0.67900000000000005</v>
       </c>
-      <c r="E5" s="16">
+      <c r="F7" s="6">
         <v>0.78500000000000003</v>
       </c>
-      <c r="F5" s="16">
+      <c r="G7" s="6">
         <v>0.80300000000000005</v>
       </c>
-      <c r="G5" s="16">
+      <c r="H7" s="6">
         <v>0.84199999999999997</v>
       </c>
-      <c r="H5" s="16">
+      <c r="I7" s="6">
         <v>0.88</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="13.9" thickTop="1">
-      <c r="A6" s="8"/>
-      <c r="B6" s="5" t="s">
+    <row r="8" spans="2:18" ht="13.9" thickTop="1">
+      <c r="B8" s="17"/>
+      <c r="C8" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="11" t="s">
-        <v>1</v>
-      </c>
-      <c r="D6" s="9">
+      <c r="D8" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="E8" s="8">
         <v>0.55300000000000005</v>
       </c>
-      <c r="E6" s="3">
+      <c r="F8" s="9">
         <v>0.69299999999999995</v>
       </c>
-      <c r="F6" s="3">
+      <c r="G8" s="9">
         <v>0.76100000000000001</v>
       </c>
-      <c r="G6" s="3">
+      <c r="H8" s="9">
         <v>0.81699999999999995</v>
       </c>
-      <c r="H6" s="3">
+      <c r="I8" s="9">
         <v>0.90200000000000002</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" ht="13.9" thickBot="1">
-      <c r="A7" s="8"/>
-      <c r="B7" s="13"/>
-      <c r="C7" s="14" t="s">
+      <c r="K8" s="13"/>
+      <c r="L8" s="23" t="s">
+        <v>12</v>
+      </c>
+      <c r="M8" s="23"/>
+      <c r="N8" s="23"/>
+      <c r="O8" s="23"/>
+      <c r="P8" s="23"/>
+      <c r="Q8" s="23"/>
+      <c r="R8" s="24"/>
+    </row>
+    <row r="9" spans="2:18" ht="13.9" thickBot="1">
+      <c r="B9" s="17"/>
+      <c r="C9" s="19"/>
+      <c r="D9" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D7" s="15">
+      <c r="E9" s="5">
         <v>0.69699999999999995</v>
       </c>
-      <c r="E7" s="16">
+      <c r="F9" s="6">
         <v>0.78300000000000003</v>
       </c>
-      <c r="F7" s="16">
+      <c r="G9" s="6">
         <v>0.80900000000000005</v>
       </c>
-      <c r="G7" s="16">
+      <c r="H9" s="6">
         <v>0.85599999999999998</v>
       </c>
-      <c r="H7" s="16">
+      <c r="I9" s="6">
         <v>0.88900000000000001</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" ht="13.9" thickTop="1">
-      <c r="A8" s="8"/>
-      <c r="B8" s="5" t="s">
+      <c r="K9" s="14"/>
+      <c r="N9" s="25" t="s">
+        <v>7</v>
+      </c>
+      <c r="O9" s="25"/>
+      <c r="P9" s="25"/>
+      <c r="Q9" s="25"/>
+      <c r="R9" s="26"/>
+    </row>
+    <row r="10" spans="2:18" ht="14.25" thickTop="1" thickBot="1">
+      <c r="B10" s="17"/>
+      <c r="C10" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="11" t="s">
-        <v>1</v>
-      </c>
-      <c r="D8" s="9">
+      <c r="D10" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="E10" s="8">
         <v>0.57699999999999996</v>
       </c>
-      <c r="E8" s="3">
+      <c r="F10" s="9">
         <v>0.67500000000000004</v>
       </c>
-      <c r="F8" s="3">
+      <c r="G10" s="9">
         <v>0.77900000000000003</v>
       </c>
-      <c r="G8" s="3">
+      <c r="H10" s="9">
         <v>0.84399999999999997</v>
       </c>
-      <c r="H8" s="3">
+      <c r="I10" s="9">
         <v>0.90200000000000002</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" ht="13.9" thickBot="1">
-      <c r="A9" s="8"/>
-      <c r="B9" s="13"/>
-      <c r="C9" s="14" t="s">
+      <c r="K10" s="14"/>
+      <c r="N10" s="12">
+        <v>0.01</v>
+      </c>
+      <c r="O10" s="12">
+        <v>0.05</v>
+      </c>
+      <c r="P10" s="12">
+        <v>0.1</v>
+      </c>
+      <c r="Q10" s="12">
+        <v>0.25</v>
+      </c>
+      <c r="R10" s="15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="2:18" ht="14.25" customHeight="1" thickTop="1" thickBot="1">
+      <c r="B11" s="17"/>
+      <c r="C11" s="19"/>
+      <c r="D11" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D9" s="15">
+      <c r="E11" s="5">
         <v>0.69099999999999995</v>
       </c>
-      <c r="E9" s="16">
+      <c r="F11" s="6">
         <v>0.78200000000000003</v>
       </c>
-      <c r="F9" s="16">
+      <c r="G11" s="6">
         <v>0.82499999999999996</v>
       </c>
-      <c r="G9" s="16">
+      <c r="H11" s="6">
         <v>0.84599999999999997</v>
       </c>
-      <c r="H9" s="16">
+      <c r="I11" s="6">
         <v>0.88</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" ht="13.9" thickTop="1">
-      <c r="A10" s="8"/>
-      <c r="B10" s="6" t="s">
+      <c r="K11" s="17" t="s">
+        <v>8</v>
+      </c>
+      <c r="L11" s="19" t="s">
+        <v>0</v>
+      </c>
+      <c r="M11" s="20"/>
+      <c r="N11" s="30" t="str">
+        <f>TEXT(AVERAGE(E5, E18, E31),"0.000")&amp;" ± "&amp;TEXT(STDEV(E5, E18, E31),"0.000")</f>
+        <v>0.636 ± 0.019</v>
+      </c>
+      <c r="O11" s="30" t="str">
+        <f t="shared" ref="O11:R11" si="0">TEXT(AVERAGE(F5, F18, F31),"0.000")&amp;" ± "&amp;TEXT(STDEV(F5, F18, F31),"0.000")</f>
+        <v>0.794 ± 0.013</v>
+      </c>
+      <c r="P11" s="30" t="str">
+        <f t="shared" si="0"/>
+        <v>0.823 ± 0.005</v>
+      </c>
+      <c r="Q11" s="30" t="str">
+        <f t="shared" si="0"/>
+        <v>0.852 ± 0.015</v>
+      </c>
+      <c r="R11" s="30" t="str">
+        <f t="shared" si="0"/>
+        <v>0.927 ± 0.003</v>
+      </c>
+    </row>
+    <row r="12" spans="2:18" ht="13.9" thickTop="1">
+      <c r="B12" s="17"/>
+      <c r="C12" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="C10" s="11" t="s">
-        <v>1</v>
-      </c>
-      <c r="D10" s="9">
+      <c r="D12" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="E12" s="8">
         <v>0.59799999999999998</v>
       </c>
-      <c r="E10" s="3">
+      <c r="F12" s="9">
         <v>0.67500000000000004</v>
       </c>
-      <c r="F10" s="3">
+      <c r="G12" s="9">
         <v>0.80700000000000005</v>
       </c>
-      <c r="G10" s="3">
+      <c r="H12" s="9">
         <v>0.82199999999999995</v>
       </c>
-      <c r="H10" s="3">
+      <c r="I12" s="9">
         <v>0.90800000000000003</v>
       </c>
-    </row>
-    <row r="11" spans="1:8">
-      <c r="A11" s="8"/>
-      <c r="B11" s="6"/>
-      <c r="C11" s="12" t="s">
+      <c r="K12" s="17"/>
+      <c r="L12" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="M12" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="N12" s="27" t="str">
+        <f>TEXT(AVERAGE(E6, E19, E32),"0.000")&amp;" ± "&amp;TEXT(STDEV(E6, E19, E32),"0.000")</f>
+        <v>0.591 ± 0.018</v>
+      </c>
+      <c r="O12" s="27" t="str">
+        <f t="shared" ref="O12:R12" si="1">TEXT(AVERAGE(F6, F19, F32),"0.000")&amp;" ± "&amp;TEXT(STDEV(F6, F19, F32),"0.000")</f>
+        <v>0.690 ± 0.040</v>
+      </c>
+      <c r="P12" s="27" t="str">
+        <f t="shared" si="1"/>
+        <v>0.780 ± 0.018</v>
+      </c>
+      <c r="Q12" s="27" t="str">
+        <f t="shared" si="1"/>
+        <v>0.824 ± 0.008</v>
+      </c>
+      <c r="R12" s="27" t="str">
+        <f t="shared" si="1"/>
+        <v>0.909 ± 0.004</v>
+      </c>
+    </row>
+    <row r="13" spans="2:18" ht="13.9" thickBot="1">
+      <c r="B13" s="18"/>
+      <c r="C13" s="22"/>
+      <c r="D13" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="D11" s="10">
+      <c r="E13" s="3">
         <v>0.77200000000000002</v>
       </c>
-      <c r="E11" s="2">
+      <c r="F13" s="2">
         <v>0.82399999999999995</v>
       </c>
-      <c r="F11" s="2">
+      <c r="G13" s="2">
         <v>0.83799999999999997</v>
       </c>
-      <c r="G11" s="2">
+      <c r="H13" s="2">
         <v>0.84699999999999998</v>
       </c>
-      <c r="H11" s="2">
+      <c r="I13" s="2">
         <v>0.88600000000000001</v>
       </c>
+      <c r="K13" s="17"/>
+      <c r="L13" s="19"/>
+      <c r="M13" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="N13" s="28" t="str">
+        <f>TEXT(AVERAGE(E7, E20, E33),"0.000")&amp;" ± "&amp;TEXT(STDEV(E7, E20, E33),"0.000")</f>
+        <v>0.714 ± 0.030</v>
+      </c>
+      <c r="O13" s="28" t="str">
+        <f t="shared" ref="O13:R14" si="2">TEXT(AVERAGE(F7, F20, F33),"0.000")&amp;" ± "&amp;TEXT(STDEV(F7, F20, F33),"0.000")</f>
+        <v>0.798 ± 0.011</v>
+      </c>
+      <c r="P13" s="28" t="str">
+        <f t="shared" si="2"/>
+        <v>0.822 ± 0.018</v>
+      </c>
+      <c r="Q13" s="28" t="str">
+        <f t="shared" si="2"/>
+        <v>0.848 ± 0.005</v>
+      </c>
+      <c r="R13" s="28" t="str">
+        <f t="shared" si="2"/>
+        <v>0.879 ± 0.002</v>
+      </c>
+    </row>
+    <row r="14" spans="2:18" ht="13.9" thickTop="1">
+      <c r="K14" s="17"/>
+      <c r="L14" s="21" t="s">
+        <v>4</v>
+      </c>
+      <c r="M14" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="N14" s="27" t="str">
+        <f t="shared" ref="N14:N19" si="3">TEXT(AVERAGE(E8, E21, E34),"0.000")&amp;" ± "&amp;TEXT(STDEV(E8, E21, E34),"0.000")</f>
+        <v>0.577 ± 0.025</v>
+      </c>
+      <c r="O14" s="27" t="str">
+        <f t="shared" si="2"/>
+        <v>0.691 ± 0.016</v>
+      </c>
+      <c r="P14" s="27" t="str">
+        <f t="shared" si="2"/>
+        <v>0.763 ± 0.003</v>
+      </c>
+      <c r="Q14" s="27" t="str">
+        <f t="shared" si="2"/>
+        <v>0.825 ± 0.010</v>
+      </c>
+      <c r="R14" s="27" t="str">
+        <f t="shared" si="2"/>
+        <v>0.907 ± 0.004</v>
+      </c>
+    </row>
+    <row r="15" spans="2:18" ht="13.9" thickBot="1">
+      <c r="B15" s="13"/>
+      <c r="C15" s="23" t="s">
+        <v>10</v>
+      </c>
+      <c r="D15" s="23"/>
+      <c r="E15" s="23"/>
+      <c r="F15" s="23"/>
+      <c r="G15" s="23"/>
+      <c r="H15" s="23"/>
+      <c r="I15" s="24"/>
+      <c r="K15" s="17"/>
+      <c r="L15" s="19"/>
+      <c r="M15" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="N15" s="28" t="str">
+        <f t="shared" si="3"/>
+        <v>0.693 ± 0.020</v>
+      </c>
+      <c r="O15" s="28" t="str">
+        <f t="shared" ref="O15:O19" si="4">TEXT(AVERAGE(F9, F22, F35),"0.000")&amp;" ± "&amp;TEXT(STDEV(F9, F22, F35),"0.000")</f>
+        <v>0.791 ± 0.010</v>
+      </c>
+      <c r="P15" s="28" t="str">
+        <f t="shared" ref="P15:P19" si="5">TEXT(AVERAGE(G9, G22, G35),"0.000")&amp;" ± "&amp;TEXT(STDEV(G9, G22, G35),"0.000")</f>
+        <v>0.820 ± 0.010</v>
+      </c>
+      <c r="Q15" s="28" t="str">
+        <f t="shared" ref="Q15:Q19" si="6">TEXT(AVERAGE(H9, H22, H35),"0.000")&amp;" ± "&amp;TEXT(STDEV(H9, H22, H35),"0.000")</f>
+        <v>0.855 ± 0.008</v>
+      </c>
+      <c r="R15" s="28" t="str">
+        <f t="shared" ref="R15:R19" si="7">TEXT(AVERAGE(I9, I22, I35),"0.000")&amp;" ± "&amp;TEXT(STDEV(I9, I22, I35),"0.000")</f>
+        <v>0.883 ± 0.008</v>
+      </c>
+    </row>
+    <row r="16" spans="2:18" ht="13.9" thickTop="1">
+      <c r="B16" s="14"/>
+      <c r="E16" s="25" t="s">
+        <v>7</v>
+      </c>
+      <c r="F16" s="25"/>
+      <c r="G16" s="25"/>
+      <c r="H16" s="25"/>
+      <c r="I16" s="26"/>
+      <c r="K16" s="17"/>
+      <c r="L16" s="21" t="s">
+        <v>5</v>
+      </c>
+      <c r="M16" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="N16" s="27" t="str">
+        <f t="shared" si="3"/>
+        <v>0.601 ± 0.041</v>
+      </c>
+      <c r="O16" s="27" t="str">
+        <f t="shared" si="4"/>
+        <v>0.658 ± 0.018</v>
+      </c>
+      <c r="P16" s="27" t="str">
+        <f t="shared" si="5"/>
+        <v>0.781 ± 0.017</v>
+      </c>
+      <c r="Q16" s="27" t="str">
+        <f t="shared" si="6"/>
+        <v>0.834 ± 0.012</v>
+      </c>
+      <c r="R16" s="27" t="str">
+        <f t="shared" si="7"/>
+        <v>0.908 ± 0.005</v>
+      </c>
+    </row>
+    <row r="17" spans="2:18" ht="13.9" thickBot="1">
+      <c r="B17" s="14"/>
+      <c r="E17" s="12">
+        <v>0.01</v>
+      </c>
+      <c r="F17" s="12">
+        <v>0.05</v>
+      </c>
+      <c r="G17" s="12">
+        <v>0.1</v>
+      </c>
+      <c r="H17" s="12">
+        <v>0.25</v>
+      </c>
+      <c r="I17" s="15">
+        <v>1</v>
+      </c>
+      <c r="K17" s="17"/>
+      <c r="L17" s="19"/>
+      <c r="M17" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="N17" s="28" t="str">
+        <f t="shared" si="3"/>
+        <v>0.701 ± 0.009</v>
+      </c>
+      <c r="O17" s="28" t="str">
+        <f t="shared" si="4"/>
+        <v>0.806 ± 0.021</v>
+      </c>
+      <c r="P17" s="28" t="str">
+        <f t="shared" si="5"/>
+        <v>0.835 ± 0.010</v>
+      </c>
+      <c r="Q17" s="28" t="str">
+        <f t="shared" si="6"/>
+        <v>0.858 ± 0.010</v>
+      </c>
+      <c r="R17" s="28" t="str">
+        <f t="shared" si="7"/>
+        <v>0.882 ± 0.002</v>
+      </c>
+    </row>
+    <row r="18" spans="2:18" ht="14.25" thickTop="1" thickBot="1">
+      <c r="B18" s="17" t="s">
+        <v>8</v>
+      </c>
+      <c r="C18" s="19" t="s">
+        <v>0</v>
+      </c>
+      <c r="D18" s="20"/>
+      <c r="E18" s="10">
+        <v>0.65600000000000003</v>
+      </c>
+      <c r="F18" s="11">
+        <v>0.80500000000000005</v>
+      </c>
+      <c r="G18" s="11">
+        <v>0.82299999999999995</v>
+      </c>
+      <c r="H18" s="11">
+        <v>0.85299999999999998</v>
+      </c>
+      <c r="I18" s="11">
+        <v>0.92500000000000004</v>
+      </c>
+      <c r="K18" s="17"/>
+      <c r="L18" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="M18" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="N18" s="27" t="str">
+        <f t="shared" si="3"/>
+        <v>0.602 ± 0.014</v>
+      </c>
+      <c r="O18" s="27" t="str">
+        <f t="shared" si="4"/>
+        <v>0.698 ± 0.021</v>
+      </c>
+      <c r="P18" s="27" t="str">
+        <f t="shared" si="5"/>
+        <v>0.774 ± 0.029</v>
+      </c>
+      <c r="Q18" s="27" t="str">
+        <f t="shared" si="6"/>
+        <v>0.826 ± 0.003</v>
+      </c>
+      <c r="R18" s="27" t="str">
+        <f t="shared" si="7"/>
+        <v>0.909 ± 0.005</v>
+      </c>
+    </row>
+    <row r="19" spans="2:18" ht="13.9" thickTop="1">
+      <c r="B19" s="17"/>
+      <c r="C19" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="D19" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="E19" s="8">
+        <v>0.61099999999999999</v>
+      </c>
+      <c r="F19" s="9">
+        <v>0.68100000000000005</v>
+      </c>
+      <c r="G19" s="9">
+        <v>0.78100000000000003</v>
+      </c>
+      <c r="H19" s="9">
+        <v>0.81599999999999995</v>
+      </c>
+      <c r="I19" s="9">
+        <v>0.90800000000000003</v>
+      </c>
+      <c r="K19" s="18"/>
+      <c r="L19" s="22"/>
+      <c r="M19" s="16" t="s">
+        <v>2</v>
+      </c>
+      <c r="N19" s="29" t="str">
+        <f t="shared" si="3"/>
+        <v>0.771 ± 0.014</v>
+      </c>
+      <c r="O19" s="29" t="str">
+        <f t="shared" si="4"/>
+        <v>0.824 ± 0.010</v>
+      </c>
+      <c r="P19" s="29" t="str">
+        <f t="shared" si="5"/>
+        <v>0.838 ± 0.003</v>
+      </c>
+      <c r="Q19" s="29" t="str">
+        <f t="shared" si="6"/>
+        <v>0.858 ± 0.010</v>
+      </c>
+      <c r="R19" s="29" t="str">
+        <f t="shared" si="7"/>
+        <v>0.883 ± 0.007</v>
+      </c>
+    </row>
+    <row r="20" spans="2:18" ht="13.9" thickBot="1">
+      <c r="B20" s="17"/>
+      <c r="C20" s="19"/>
+      <c r="D20" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E20" s="5">
+        <v>0.73399999999999999</v>
+      </c>
+      <c r="F20" s="6">
+        <v>0.80500000000000005</v>
+      </c>
+      <c r="G20" s="6">
+        <v>0.83799999999999997</v>
+      </c>
+      <c r="H20" s="6">
+        <v>0.85</v>
+      </c>
+      <c r="I20" s="6">
+        <v>0.877</v>
+      </c>
+    </row>
+    <row r="21" spans="2:18" ht="13.9" thickTop="1">
+      <c r="B21" s="17"/>
+      <c r="C21" s="21" t="s">
+        <v>4</v>
+      </c>
+      <c r="D21" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="E21" s="8">
+        <v>0.57699999999999996</v>
+      </c>
+      <c r="F21" s="9">
+        <v>0.67400000000000004</v>
+      </c>
+      <c r="G21" s="9">
+        <v>0.76600000000000001</v>
+      </c>
+      <c r="H21" s="9">
+        <v>0.82199999999999995</v>
+      </c>
+      <c r="I21" s="9">
+        <v>0.91</v>
+      </c>
+    </row>
+    <row r="22" spans="2:18" ht="13.9" thickBot="1">
+      <c r="B22" s="17"/>
+      <c r="C22" s="19"/>
+      <c r="D22" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E22" s="5">
+        <v>0.71</v>
+      </c>
+      <c r="F22" s="6">
+        <v>0.80200000000000005</v>
+      </c>
+      <c r="G22" s="6">
+        <v>0.82599999999999996</v>
+      </c>
+      <c r="H22" s="6">
+        <v>0.84599999999999997</v>
+      </c>
+      <c r="I22" s="6">
+        <v>0.874</v>
+      </c>
+    </row>
+    <row r="23" spans="2:18" ht="13.9" thickTop="1">
+      <c r="B23" s="17"/>
+      <c r="C23" s="21" t="s">
+        <v>5</v>
+      </c>
+      <c r="D23" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="E23" s="8">
+        <v>0.64900000000000002</v>
+      </c>
+      <c r="F23" s="9">
+        <v>0.63900000000000001</v>
+      </c>
+      <c r="G23" s="9">
+        <v>0.79900000000000004</v>
+      </c>
+      <c r="H23" s="9">
+        <v>0.82099999999999995</v>
+      </c>
+      <c r="I23" s="9">
+        <v>0.91100000000000003</v>
+      </c>
+    </row>
+    <row r="24" spans="2:18" ht="13.9" thickBot="1">
+      <c r="B24" s="17"/>
+      <c r="C24" s="19"/>
+      <c r="D24" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E24" s="5">
+        <v>0.70199999999999996</v>
+      </c>
+      <c r="F24" s="6">
+        <v>0.81799999999999995</v>
+      </c>
+      <c r="G24" s="6">
+        <v>0.83499999999999996</v>
+      </c>
+      <c r="H24" s="6">
+        <v>0.86199999999999999</v>
+      </c>
+      <c r="I24" s="6">
+        <v>0.88300000000000001</v>
+      </c>
+    </row>
+    <row r="25" spans="2:18" ht="13.9" thickTop="1">
+      <c r="B25" s="17"/>
+      <c r="C25" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="D25" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="E25" s="8">
+        <v>0.61799999999999999</v>
+      </c>
+      <c r="F25" s="9">
+        <v>0.71499999999999997</v>
+      </c>
+      <c r="G25" s="9">
+        <v>0.76500000000000001</v>
+      </c>
+      <c r="H25" s="9">
+        <v>0.82699999999999996</v>
+      </c>
+      <c r="I25" s="9">
+        <v>0.91400000000000003</v>
+      </c>
+    </row>
+    <row r="26" spans="2:18">
+      <c r="B26" s="18"/>
+      <c r="C26" s="22"/>
+      <c r="D26" s="16" t="s">
+        <v>2</v>
+      </c>
+      <c r="E26" s="3">
+        <v>0.78400000000000003</v>
+      </c>
+      <c r="F26" s="2">
+        <v>0.81399999999999995</v>
+      </c>
+      <c r="G26" s="2">
+        <v>0.84099999999999997</v>
+      </c>
+      <c r="H26" s="2">
+        <v>0.85899999999999999</v>
+      </c>
+      <c r="I26" s="2">
+        <v>0.875</v>
+      </c>
+    </row>
+    <row r="28" spans="2:18">
+      <c r="B28" s="13"/>
+      <c r="C28" s="23" t="s">
+        <v>11</v>
+      </c>
+      <c r="D28" s="23"/>
+      <c r="E28" s="23"/>
+      <c r="F28" s="23"/>
+      <c r="G28" s="23"/>
+      <c r="H28" s="23"/>
+      <c r="I28" s="24"/>
+    </row>
+    <row r="29" spans="2:18">
+      <c r="B29" s="14"/>
+      <c r="E29" s="25" t="s">
+        <v>7</v>
+      </c>
+      <c r="F29" s="25"/>
+      <c r="G29" s="25"/>
+      <c r="H29" s="25"/>
+      <c r="I29" s="26"/>
+    </row>
+    <row r="30" spans="2:18" ht="13.9" thickBot="1">
+      <c r="B30" s="14"/>
+      <c r="E30" s="12">
+        <v>0.01</v>
+      </c>
+      <c r="F30" s="12">
+        <v>0.05</v>
+      </c>
+      <c r="G30" s="12">
+        <v>0.1</v>
+      </c>
+      <c r="H30" s="12">
+        <v>0.25</v>
+      </c>
+      <c r="I30" s="15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="2:18" ht="14.25" thickTop="1" thickBot="1">
+      <c r="B31" s="17" t="s">
+        <v>8</v>
+      </c>
+      <c r="C31" s="19" t="s">
+        <v>0</v>
+      </c>
+      <c r="D31" s="20"/>
+      <c r="E31" s="10">
+        <v>0.63300000000000001</v>
+      </c>
+      <c r="F31" s="11">
+        <v>0.79600000000000004</v>
+      </c>
+      <c r="G31" s="11">
+        <v>0.82799999999999996</v>
+      </c>
+      <c r="H31" s="11">
+        <v>0.86599999999999999</v>
+      </c>
+      <c r="I31" s="11">
+        <v>0.93</v>
+      </c>
+    </row>
+    <row r="32" spans="2:18" ht="13.9" thickTop="1">
+      <c r="B32" s="17"/>
+      <c r="C32" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="D32" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="E32" s="8">
+        <v>0.58299999999999996</v>
+      </c>
+      <c r="F32" s="9">
+        <v>0.73399999999999999</v>
+      </c>
+      <c r="G32" s="9">
+        <v>0.79700000000000004</v>
+      </c>
+      <c r="H32" s="9">
+        <v>0.83099999999999996</v>
+      </c>
+      <c r="I32" s="9">
+        <v>0.90600000000000003</v>
+      </c>
+    </row>
+    <row r="33" spans="2:9" ht="13.9" thickBot="1">
+      <c r="B33" s="17"/>
+      <c r="C33" s="19"/>
+      <c r="D33" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E33" s="5">
+        <v>0.72899999999999998</v>
+      </c>
+      <c r="F33" s="6">
+        <v>0.80300000000000005</v>
+      </c>
+      <c r="G33" s="6">
+        <v>0.82599999999999996</v>
+      </c>
+      <c r="H33" s="6">
+        <v>0.85099999999999998</v>
+      </c>
+      <c r="I33" s="6">
+        <v>0.879</v>
+      </c>
+    </row>
+    <row r="34" spans="2:9" ht="13.9" thickTop="1">
+      <c r="B34" s="17"/>
+      <c r="C34" s="21" t="s">
+        <v>4</v>
+      </c>
+      <c r="D34" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="E34" s="8">
+        <v>0.60199999999999998</v>
+      </c>
+      <c r="F34" s="9">
+        <v>0.70599999999999996</v>
+      </c>
+      <c r="G34" s="9">
+        <v>0.76100000000000001</v>
+      </c>
+      <c r="H34" s="9">
+        <v>0.83599999999999997</v>
+      </c>
+      <c r="I34" s="9">
+        <v>0.90900000000000003</v>
+      </c>
+    </row>
+    <row r="35" spans="2:9" ht="13.9" thickBot="1">
+      <c r="B35" s="17"/>
+      <c r="C35" s="19"/>
+      <c r="D35" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E35" s="5">
+        <v>0.67100000000000004</v>
+      </c>
+      <c r="F35" s="6">
+        <v>0.78800000000000003</v>
+      </c>
+      <c r="G35" s="6">
+        <v>0.82499999999999996</v>
+      </c>
+      <c r="H35" s="6">
+        <v>0.86199999999999999</v>
+      </c>
+      <c r="I35" s="6">
+        <v>0.88500000000000001</v>
+      </c>
+    </row>
+    <row r="36" spans="2:9" ht="13.9" thickTop="1">
+      <c r="B36" s="17"/>
+      <c r="C36" s="21" t="s">
+        <v>5</v>
+      </c>
+      <c r="D36" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="E36" s="8">
+        <v>0.57799999999999996</v>
+      </c>
+      <c r="F36" s="9">
+        <v>0.66100000000000003</v>
+      </c>
+      <c r="G36" s="9">
+        <v>0.76600000000000001</v>
+      </c>
+      <c r="H36" s="9">
+        <v>0.83599999999999997</v>
+      </c>
+      <c r="I36" s="9">
+        <v>0.91100000000000003</v>
+      </c>
+    </row>
+    <row r="37" spans="2:9" ht="13.9" thickBot="1">
+      <c r="B37" s="17"/>
+      <c r="C37" s="19"/>
+      <c r="D37" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E37" s="5">
+        <v>0.70899999999999996</v>
+      </c>
+      <c r="F37" s="6">
+        <v>0.81699999999999995</v>
+      </c>
+      <c r="G37" s="6">
+        <v>0.84399999999999997</v>
+      </c>
+      <c r="H37" s="6">
+        <v>0.86499999999999999</v>
+      </c>
+      <c r="I37" s="6">
+        <v>0.88300000000000001</v>
+      </c>
+    </row>
+    <row r="38" spans="2:9" ht="13.9" thickTop="1">
+      <c r="B38" s="17"/>
+      <c r="C38" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="D38" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="E38" s="8">
+        <v>0.59</v>
+      </c>
+      <c r="F38" s="9">
+        <v>0.70299999999999996</v>
+      </c>
+      <c r="G38" s="9">
+        <v>0.751</v>
+      </c>
+      <c r="H38" s="9">
+        <v>0.82799999999999996</v>
+      </c>
+      <c r="I38" s="9">
+        <v>0.90500000000000003</v>
+      </c>
+    </row>
+    <row r="39" spans="2:9">
+      <c r="B39" s="18"/>
+      <c r="C39" s="22"/>
+      <c r="D39" s="16" t="s">
+        <v>2</v>
+      </c>
+      <c r="E39" s="3">
+        <v>0.75600000000000001</v>
+      </c>
+      <c r="F39" s="2">
+        <v>0.83399999999999996</v>
+      </c>
+      <c r="G39" s="2">
+        <v>0.83599999999999997</v>
+      </c>
+      <c r="H39" s="2">
+        <v>0.86699999999999999</v>
+      </c>
+      <c r="I39" s="2">
+        <v>0.88900000000000001</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="B8:B9"/>
-    <mergeCell ref="B10:B11"/>
-    <mergeCell ref="D1:H1"/>
-    <mergeCell ref="A3:A11"/>
+  <mergeCells count="32">
+    <mergeCell ref="E29:I29"/>
+    <mergeCell ref="B31:B39"/>
+    <mergeCell ref="C31:D31"/>
+    <mergeCell ref="C32:C33"/>
+    <mergeCell ref="C34:C35"/>
+    <mergeCell ref="C36:C37"/>
+    <mergeCell ref="C38:C39"/>
+    <mergeCell ref="B5:B13"/>
+    <mergeCell ref="E16:I16"/>
+    <mergeCell ref="B18:B26"/>
+    <mergeCell ref="C18:D18"/>
+    <mergeCell ref="C19:C20"/>
+    <mergeCell ref="C21:C22"/>
+    <mergeCell ref="C23:C24"/>
+    <mergeCell ref="C25:C26"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="C6:C7"/>
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="C10:C11"/>
+    <mergeCell ref="C12:C13"/>
+    <mergeCell ref="L8:R8"/>
+    <mergeCell ref="N9:R9"/>
+    <mergeCell ref="C2:I2"/>
+    <mergeCell ref="C15:I15"/>
+    <mergeCell ref="C28:I28"/>
+    <mergeCell ref="L12:L13"/>
+    <mergeCell ref="E3:I3"/>
+    <mergeCell ref="K11:K19"/>
+    <mergeCell ref="L11:M11"/>
+    <mergeCell ref="L14:L15"/>
+    <mergeCell ref="L16:L17"/>
+    <mergeCell ref="L18:L19"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>